<commit_message>
Add Appium mobile E2E test suite, 305 test cases Excel report, and GitHub Actions workflow
</commit_message>
<xml_diff>
--- a/selenium-tests/selenium_test_report.xlsx
+++ b/selenium-tests/selenium_test_report.xlsx
@@ -429,7 +429,7 @@
         <v>Target Application URL</v>
       </c>
       <c r="B4" t="str">
-        <v>http://localhost:3000</v>
+        <v>https://toolshare-production-e02e.up.railway.app</v>
       </c>
     </row>
     <row r="5">
@@ -485,7 +485,7 @@
         <v>Report Generated At</v>
       </c>
       <c r="B11" t="str">
-        <v>23/7/2026, 1:36:38 pm</v>
+        <v>23/7/2026, 1:58:59 pm</v>
       </c>
     </row>
   </sheetData>

</xml_diff>